<commit_message>
We zijn goed op weg :) (It is not saturday, I swear \('_')/)
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/demand_scenarios111.xlsx
+++ b/study_case_model/scenario_variables/demand_scenarios111.xlsx
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>25.85282053282582</v>
+        <v>25852.82053282582</v>
       </c>
     </row>
     <row r="3">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2.872535614758425</v>
+        <v>2872.535614758425</v>
       </c>
     </row>
     <row r="4">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>23.96301774121611</v>
+        <v>23963.01774121611</v>
       </c>
     </row>
     <row r="6">
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>23.88613122860416</v>
+        <v>23886.13122860416</v>
       </c>
     </row>
     <row r="9">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>5.971532807151039</v>
+        <v>5971.532807151039</v>
       </c>
     </row>
     <row r="11">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>72.84544784612038</v>
+        <v>72845.44784612038</v>
       </c>
     </row>
     <row r="12">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>11.62192484478749</v>
+        <v>11621.92484478749</v>
       </c>
     </row>
     <row r="15">

</xml_diff>